<commit_message>
Publish fund screening framework page and update project cards
- New fund-screening.html: 3-layer methodology, 5-factor scoring engine,
  80 Indian equity funds across 4 SEBI categories
- New fund-screening.css: scoped stylesheet for framework page
- index.html: project card updated (In Progress → Published, revised
  description, added View Methodology link); Currently section updated
  (50% → 100% complete, detail text corrected)
- Updated Excel models: fund-screening-model.xlsx, angel-one-model.xlsx
- Added fund screening data files and methodology PDFs
- CSS updates: equity-research.css, company-model.css, horizon2040.css,
  signals.css, styles.css
</commit_message>
<xml_diff>
--- a/projects/angel-one/angel-one-model.xlsx
+++ b/projects/angel-one/angel-one-model.xlsx
@@ -221,7 +221,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -243,11 +243,104 @@
         <color rgb="00C0C0C0"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C0C0C0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C0C0C0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C0C0C0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C0C0C0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C0C0C0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C0C0C0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C0C0C0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C0C0C0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C0C0C0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C0C0C0"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C0C0C0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00C0C0C0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00C0C0C0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C0C0C0"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00C0C0C0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -462,6 +555,15 @@
     <xf numFmtId="0" fontId="16" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -875,6 +977,16 @@
           <t>ANGEL ONE LTD (NSE: ANGELONE) — 3-Statement Financial Model</t>
         </is>
       </c>
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="72" t="n"/>
+      <c r="G1" s="72" t="n"/>
+      <c r="H1" s="72" t="n"/>
+      <c r="I1" s="72" t="n"/>
+      <c r="J1" s="72" t="n"/>
+      <c r="K1" s="73" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -941,6 +1053,16 @@
           <t>KEY ASSUMPTIONS (FY25E–FY29E — OVERRIDE THESE WITH YOUR VIEWS)</t>
         </is>
       </c>
+      <c r="B5" s="72" t="n"/>
+      <c r="C5" s="72" t="n"/>
+      <c r="D5" s="72" t="n"/>
+      <c r="E5" s="72" t="n"/>
+      <c r="F5" s="72" t="n"/>
+      <c r="G5" s="72" t="n"/>
+      <c r="H5" s="72" t="n"/>
+      <c r="I5" s="72" t="n"/>
+      <c r="J5" s="72" t="n"/>
+      <c r="K5" s="73" t="n"/>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
@@ -1221,19 +1343,19 @@
         </is>
       </c>
       <c r="F12" s="9" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>0.335</v>
+      </c>
+      <c r="H12" s="9" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="I12" s="9" t="n">
+        <v>0.365</v>
+      </c>
+      <c r="J12" s="9" t="n">
         <v>0.38</v>
-      </c>
-      <c r="G12" s="9" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="H12" s="9" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="I12" s="9" t="n">
-        <v>0.43</v>
-      </c>
-      <c r="J12" s="9" t="n">
-        <v>0.44</v>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1">
@@ -1410,6 +1532,16 @@
           <t>INCOME STATEMENT</t>
         </is>
       </c>
+      <c r="B18" s="72" t="n"/>
+      <c r="C18" s="72" t="n"/>
+      <c r="D18" s="72" t="n"/>
+      <c r="E18" s="72" t="n"/>
+      <c r="F18" s="72" t="n"/>
+      <c r="G18" s="72" t="n"/>
+      <c r="H18" s="72" t="n"/>
+      <c r="I18" s="72" t="n"/>
+      <c r="J18" s="72" t="n"/>
+      <c r="K18" s="73" t="n"/>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="11" t="inlineStr">
@@ -1417,10 +1549,18 @@
           <t xml:space="preserve">  Brokerage Revenue</t>
         </is>
       </c>
-      <c r="B19" s="12" t="n"/>
-      <c r="C19" s="12" t="n"/>
-      <c r="D19" s="12" t="n"/>
-      <c r="E19" s="12" t="n"/>
+      <c r="B19" s="12" t="n">
+        <v>9085.41</v>
+      </c>
+      <c r="C19" s="12" t="n">
+        <v>16792.29</v>
+      </c>
+      <c r="D19" s="12" t="n">
+        <v>20805</v>
+      </c>
+      <c r="E19" s="12" t="n">
+        <v>29225</v>
+      </c>
       <c r="F19" s="13">
         <f>E19*(1+F6)*(1+F7)</f>
         <v/>
@@ -1448,10 +1588,18 @@
           <t xml:space="preserve">  Distribution Revenue</t>
         </is>
       </c>
-      <c r="B20" s="12" t="n"/>
-      <c r="C20" s="12" t="n"/>
-      <c r="D20" s="12" t="n"/>
-      <c r="E20" s="12" t="n"/>
+      <c r="B20" s="12" t="n">
+        <v>156.12</v>
+      </c>
+      <c r="C20" s="12" t="n">
+        <v>323.72</v>
+      </c>
+      <c r="D20" s="12" t="n">
+        <v>313</v>
+      </c>
+      <c r="E20" s="12" t="n">
+        <v>452</v>
+      </c>
       <c r="F20" s="13">
         <f>E20*(1+F9)</f>
         <v/>
@@ -1479,10 +1627,18 @@
           <t xml:space="preserve">  DP &amp; Other Revenue</t>
         </is>
       </c>
-      <c r="B21" s="12" t="n"/>
-      <c r="C21" s="12" t="n"/>
-      <c r="D21" s="12" t="n"/>
-      <c r="E21" s="12" t="n"/>
+      <c r="B21" s="12" t="n">
+        <v>1963.69</v>
+      </c>
+      <c r="C21" s="12" t="n">
+        <v>2606.45</v>
+      </c>
+      <c r="D21" s="12" t="n">
+        <v>3898.13</v>
+      </c>
+      <c r="E21" s="12" t="n">
+        <v>5262.05</v>
+      </c>
       <c r="F21" s="13">
         <f>E21*(1+F6)</f>
         <v/>
@@ -1510,10 +1666,18 @@
           <t xml:space="preserve">  MTF Interest Income</t>
         </is>
       </c>
-      <c r="B22" s="12" t="n"/>
-      <c r="C22" s="12" t="n"/>
-      <c r="D22" s="12" t="n"/>
-      <c r="E22" s="12" t="n"/>
+      <c r="B22" s="12" t="n">
+        <v>1692.21</v>
+      </c>
+      <c r="C22" s="12" t="n">
+        <v>3328.24</v>
+      </c>
+      <c r="D22" s="12" t="n">
+        <v>5195.05</v>
+      </c>
+      <c r="E22" s="12" t="n">
+        <v>7858.83</v>
+      </c>
       <c r="F22" s="13">
         <f>E22*(1+F10)</f>
         <v/>
@@ -1541,10 +1705,18 @@
           <t>Total Revenue</t>
         </is>
       </c>
-      <c r="B23" s="15" t="n"/>
-      <c r="C23" s="15" t="n"/>
-      <c r="D23" s="15" t="n"/>
-      <c r="E23" s="15" t="n"/>
+      <c r="B23" s="15" t="n">
+        <v>12897.43</v>
+      </c>
+      <c r="C23" s="15" t="n">
+        <v>23050.7</v>
+      </c>
+      <c r="D23" s="15" t="n">
+        <v>30211.18</v>
+      </c>
+      <c r="E23" s="15" t="n">
+        <v>42797.88</v>
+      </c>
       <c r="F23" s="16">
         <f>F19+F20+F21+F22</f>
         <v/>
@@ -1573,10 +1745,18 @@
           <t xml:space="preserve">  Employee Costs</t>
         </is>
       </c>
-      <c r="B25" s="12" t="n"/>
-      <c r="C25" s="12" t="n"/>
-      <c r="D25" s="12" t="n"/>
-      <c r="E25" s="12" t="n"/>
+      <c r="B25" s="12" t="n">
+        <v>1644.19</v>
+      </c>
+      <c r="C25" s="12" t="n">
+        <v>2808.99</v>
+      </c>
+      <c r="D25" s="12" t="n">
+        <v>3979.02</v>
+      </c>
+      <c r="E25" s="12" t="n">
+        <v>5584.62</v>
+      </c>
       <c r="F25" s="13" t="n"/>
       <c r="G25" s="13" t="n"/>
       <c r="H25" s="13" t="n"/>
@@ -1589,10 +1769,18 @@
           <t xml:space="preserve">  Technology Costs</t>
         </is>
       </c>
-      <c r="B26" s="12" t="n"/>
-      <c r="C26" s="12" t="n"/>
-      <c r="D26" s="12" t="n"/>
-      <c r="E26" s="12" t="n"/>
+      <c r="B26" s="12" t="n">
+        <v>357</v>
+      </c>
+      <c r="C26" s="12" t="n">
+        <v>694</v>
+      </c>
+      <c r="D26" s="12" t="n">
+        <v>1250</v>
+      </c>
+      <c r="E26" s="12" t="n">
+        <v>2252</v>
+      </c>
       <c r="F26" s="13" t="n"/>
       <c r="G26" s="13" t="n"/>
       <c r="H26" s="13" t="n"/>
@@ -1605,10 +1793,18 @@
           <t xml:space="preserve">  Marketing Costs</t>
         </is>
       </c>
-      <c r="B27" s="12" t="n"/>
-      <c r="C27" s="12" t="n"/>
-      <c r="D27" s="12" t="n"/>
-      <c r="E27" s="12" t="n"/>
+      <c r="B27" s="12" t="n">
+        <v>1277</v>
+      </c>
+      <c r="C27" s="12" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D27" s="12" t="n">
+        <v>3800</v>
+      </c>
+      <c r="E27" s="12" t="n">
+        <v>6864</v>
+      </c>
       <c r="F27" s="13" t="n"/>
       <c r="G27" s="13" t="n"/>
       <c r="H27" s="13" t="n"/>
@@ -1621,10 +1817,18 @@
           <t xml:space="preserve">  Other OpEx</t>
         </is>
       </c>
-      <c r="B28" s="12" t="n"/>
-      <c r="C28" s="12" t="n"/>
-      <c r="D28" s="12" t="n"/>
-      <c r="E28" s="12" t="n"/>
+      <c r="B28" s="12" t="n">
+        <v>4866.88</v>
+      </c>
+      <c r="C28" s="12" t="n">
+        <v>7272.72</v>
+      </c>
+      <c r="D28" s="12" t="n">
+        <v>8066.19</v>
+      </c>
+      <c r="E28" s="12" t="n">
+        <v>11107.71</v>
+      </c>
       <c r="F28" s="13" t="n"/>
       <c r="G28" s="13" t="n"/>
       <c r="H28" s="13" t="n"/>
@@ -1637,10 +1841,18 @@
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="B29" s="15" t="n"/>
-      <c r="C29" s="15" t="n"/>
-      <c r="D29" s="15" t="n"/>
-      <c r="E29" s="15" t="n"/>
+      <c r="B29" s="15" t="n">
+        <v>4752.36</v>
+      </c>
+      <c r="C29" s="15" t="n">
+        <v>9274.99</v>
+      </c>
+      <c r="D29" s="15" t="n">
+        <v>13115.97</v>
+      </c>
+      <c r="E29" s="15" t="n">
+        <v>16989.55</v>
+      </c>
       <c r="F29" s="16">
         <f>F23*F12</f>
         <v/>
@@ -1668,10 +1880,18 @@
           <t>EBITDA Margin (%)</t>
         </is>
       </c>
-      <c r="B30" s="9" t="n"/>
-      <c r="C30" s="9" t="n"/>
-      <c r="D30" s="9" t="n"/>
-      <c r="E30" s="9" t="n"/>
+      <c r="B30" s="9" t="n">
+        <v>0.36847</v>
+      </c>
+      <c r="C30" s="9" t="n">
+        <v>0.40237</v>
+      </c>
+      <c r="D30" s="9" t="n">
+        <v>0.43414</v>
+      </c>
+      <c r="E30" s="9" t="n">
+        <v>0.39697</v>
+      </c>
       <c r="F30" s="17">
         <f>F29/F23</f>
         <v/>
@@ -1699,10 +1919,18 @@
           <t xml:space="preserve">  D&amp;A</t>
         </is>
       </c>
-      <c r="B31" s="12" t="n"/>
-      <c r="C31" s="12" t="n"/>
-      <c r="D31" s="12" t="n"/>
-      <c r="E31" s="12" t="n"/>
+      <c r="B31" s="12" t="n">
+        <v>174.24</v>
+      </c>
+      <c r="C31" s="12" t="n">
+        <v>188.41</v>
+      </c>
+      <c r="D31" s="12" t="n">
+        <v>302.64</v>
+      </c>
+      <c r="E31" s="12" t="n">
+        <v>493.3</v>
+      </c>
       <c r="F31" s="13">
         <f>F23*F13</f>
         <v/>
@@ -1730,10 +1958,18 @@
           <t>EBIT</t>
         </is>
       </c>
-      <c r="B32" s="15" t="n"/>
-      <c r="C32" s="15" t="n"/>
-      <c r="D32" s="15" t="n"/>
-      <c r="E32" s="15" t="n"/>
+      <c r="B32" s="15" t="n">
+        <v>4578.12</v>
+      </c>
+      <c r="C32" s="15" t="n">
+        <v>9086.58</v>
+      </c>
+      <c r="D32" s="15" t="n">
+        <v>12813.33</v>
+      </c>
+      <c r="E32" s="15" t="n">
+        <v>16496.25</v>
+      </c>
       <c r="F32" s="16">
         <f>F29-F31</f>
         <v/>
@@ -1761,10 +1997,18 @@
           <t xml:space="preserve">  Finance Costs</t>
         </is>
       </c>
-      <c r="B33" s="12" t="n"/>
-      <c r="C33" s="12" t="n"/>
-      <c r="D33" s="12" t="n"/>
-      <c r="E33" s="12" t="n"/>
+      <c r="B33" s="12" t="n">
+        <v>596.33</v>
+      </c>
+      <c r="C33" s="12" t="n">
+        <v>721.47</v>
+      </c>
+      <c r="D33" s="12" t="n">
+        <v>895.15</v>
+      </c>
+      <c r="E33" s="12" t="n">
+        <v>1359.45</v>
+      </c>
       <c r="F33" s="12" t="inlineStr"/>
       <c r="G33" s="12" t="inlineStr"/>
       <c r="H33" s="12" t="inlineStr"/>
@@ -1777,10 +2021,18 @@
           <t>PBT</t>
         </is>
       </c>
-      <c r="B34" s="15" t="n"/>
-      <c r="C34" s="15" t="n"/>
-      <c r="D34" s="15" t="n"/>
-      <c r="E34" s="15" t="n"/>
+      <c r="B34" s="15" t="n">
+        <v>3981.79</v>
+      </c>
+      <c r="C34" s="15" t="n">
+        <v>8367.110000000001</v>
+      </c>
+      <c r="D34" s="15" t="n">
+        <v>11918.18</v>
+      </c>
+      <c r="E34" s="15" t="n">
+        <v>15137.3</v>
+      </c>
       <c r="F34" s="16">
         <f>F32-F33</f>
         <v/>
@@ -1808,10 +2060,18 @@
           <t xml:space="preserve">  Tax</t>
         </is>
       </c>
-      <c r="B35" s="12" t="n"/>
-      <c r="C35" s="12" t="n"/>
-      <c r="D35" s="12" t="n"/>
-      <c r="E35" s="12" t="n"/>
+      <c r="B35" s="12" t="n">
+        <v>1077.82</v>
+      </c>
+      <c r="C35" s="12" t="n">
+        <v>2116.55</v>
+      </c>
+      <c r="D35" s="12" t="n">
+        <v>3016.26</v>
+      </c>
+      <c r="E35" s="12" t="n">
+        <v>3881.41</v>
+      </c>
       <c r="F35" s="13">
         <f>F34*F14</f>
         <v/>
@@ -1839,10 +2099,18 @@
           <t>PAT (Net Profit)</t>
         </is>
       </c>
-      <c r="B36" s="15" t="n"/>
-      <c r="C36" s="15" t="n"/>
-      <c r="D36" s="15" t="n"/>
-      <c r="E36" s="15" t="n"/>
+      <c r="B36" s="15" t="n">
+        <v>2903.97</v>
+      </c>
+      <c r="C36" s="15" t="n">
+        <v>6248.05</v>
+      </c>
+      <c r="D36" s="15" t="n">
+        <v>8899.540000000001</v>
+      </c>
+      <c r="E36" s="15" t="n">
+        <v>11255.28</v>
+      </c>
       <c r="F36" s="16">
         <f>F34-F35</f>
         <v/>
@@ -1870,10 +2138,18 @@
           <t>PAT Margin (%)</t>
         </is>
       </c>
-      <c r="B37" s="9" t="n"/>
-      <c r="C37" s="9" t="n"/>
-      <c r="D37" s="9" t="n"/>
-      <c r="E37" s="9" t="n"/>
+      <c r="B37" s="9" t="n">
+        <v>0.22516</v>
+      </c>
+      <c r="C37" s="9" t="n">
+        <v>0.27106</v>
+      </c>
+      <c r="D37" s="9" t="n">
+        <v>0.29458</v>
+      </c>
+      <c r="E37" s="9" t="n">
+        <v>0.26299</v>
+      </c>
       <c r="F37" s="17">
         <f>F36/F23</f>
         <v/>
@@ -1901,10 +2177,18 @@
           <t>EPS (₹)</t>
         </is>
       </c>
-      <c r="B38" s="9" t="n"/>
-      <c r="C38" s="9" t="n"/>
-      <c r="D38" s="9" t="n"/>
-      <c r="E38" s="9" t="n"/>
+      <c r="B38" s="9" t="n">
+        <v>3.749</v>
+      </c>
+      <c r="C38" s="9" t="n">
+        <v>7.444</v>
+      </c>
+      <c r="D38" s="9" t="n">
+        <v>10.509</v>
+      </c>
+      <c r="E38" s="9" t="n">
+        <v>13.181</v>
+      </c>
       <c r="F38" s="18">
         <f>F36/Assumptions!B2*1000000</f>
         <v/>
@@ -1932,6 +2216,16 @@
           <t>BALANCE SHEET</t>
         </is>
       </c>
+      <c r="B41" s="72" t="n"/>
+      <c r="C41" s="72" t="n"/>
+      <c r="D41" s="72" t="n"/>
+      <c r="E41" s="72" t="n"/>
+      <c r="F41" s="72" t="n"/>
+      <c r="G41" s="72" t="n"/>
+      <c r="H41" s="72" t="n"/>
+      <c r="I41" s="72" t="n"/>
+      <c r="J41" s="72" t="n"/>
+      <c r="K41" s="73" t="n"/>
     </row>
     <row r="42" ht="16" customHeight="1">
       <c r="A42" s="14" t="inlineStr">
@@ -1955,10 +2249,18 @@
           <t xml:space="preserve">  Fixed Assets (net)</t>
         </is>
       </c>
-      <c r="B43" s="12" t="n"/>
-      <c r="C43" s="12" t="n"/>
-      <c r="D43" s="12" t="n"/>
-      <c r="E43" s="12" t="n"/>
+      <c r="B43" s="12" t="n">
+        <v>1002.96</v>
+      </c>
+      <c r="C43" s="12" t="n">
+        <v>1638.22</v>
+      </c>
+      <c r="D43" s="12" t="n">
+        <v>3065.75</v>
+      </c>
+      <c r="E43" s="12" t="n">
+        <v>4093.78</v>
+      </c>
       <c r="F43" s="13">
         <f>E43+F23*F15-F31</f>
         <v/>
@@ -1986,10 +2288,18 @@
           <t xml:space="preserve">  Investments &amp; Securities</t>
         </is>
       </c>
-      <c r="B44" s="12" t="n"/>
-      <c r="C44" s="12" t="n"/>
-      <c r="D44" s="12" t="n"/>
-      <c r="E44" s="12" t="n"/>
+      <c r="B44" s="12" t="n">
+        <v>329.79</v>
+      </c>
+      <c r="C44" s="12" t="n">
+        <v>186.52</v>
+      </c>
+      <c r="D44" s="12" t="n">
+        <v>1094.74</v>
+      </c>
+      <c r="E44" s="12" t="n">
+        <v>0</v>
+      </c>
       <c r="F44" s="13" t="n"/>
       <c r="G44" s="13" t="n"/>
       <c r="H44" s="13" t="n"/>
@@ -2002,10 +2312,18 @@
           <t xml:space="preserve">  Client Receivables</t>
         </is>
       </c>
-      <c r="B45" s="12" t="n"/>
-      <c r="C45" s="12" t="n"/>
-      <c r="D45" s="12" t="n"/>
-      <c r="E45" s="12" t="n"/>
+      <c r="B45" s="12" t="n">
+        <v>12905.55</v>
+      </c>
+      <c r="C45" s="12" t="n">
+        <v>19228.24</v>
+      </c>
+      <c r="D45" s="12" t="n">
+        <v>13800.67</v>
+      </c>
+      <c r="E45" s="12" t="n">
+        <v>19710.7</v>
+      </c>
       <c r="F45" s="13">
         <f>F23*F16</f>
         <v/>
@@ -2033,10 +2351,18 @@
           <t xml:space="preserve">  Other Current Assets</t>
         </is>
       </c>
-      <c r="B46" s="12" t="n"/>
-      <c r="C46" s="12" t="n"/>
-      <c r="D46" s="12" t="n"/>
-      <c r="E46" s="12" t="n"/>
+      <c r="B46" s="12" t="n">
+        <v>14578.38</v>
+      </c>
+      <c r="C46" s="12" t="n">
+        <v>2396.88</v>
+      </c>
+      <c r="D46" s="12" t="n">
+        <v>1979.4</v>
+      </c>
+      <c r="E46" s="12" t="n">
+        <v>10129.81</v>
+      </c>
       <c r="F46" s="13" t="n"/>
       <c r="G46" s="13" t="n"/>
       <c r="H46" s="13" t="n"/>
@@ -2049,10 +2375,18 @@
           <t xml:space="preserve">  Cash &amp; Cash Equivalents</t>
         </is>
       </c>
-      <c r="B47" s="12" t="n"/>
-      <c r="C47" s="12" t="n"/>
-      <c r="D47" s="12" t="n"/>
-      <c r="E47" s="12" t="n"/>
+      <c r="B47" s="12" t="n">
+        <v>18510.51</v>
+      </c>
+      <c r="C47" s="12" t="n">
+        <v>48749.57</v>
+      </c>
+      <c r="D47" s="12" t="n">
+        <v>54910.83</v>
+      </c>
+      <c r="E47" s="12" t="n">
+        <v>98442.94</v>
+      </c>
       <c r="F47" s="13" t="n"/>
       <c r="G47" s="13" t="n"/>
       <c r="H47" s="13" t="n"/>
@@ -2065,10 +2399,18 @@
           <t>Total Assets</t>
         </is>
       </c>
-      <c r="B48" s="19" t="n"/>
-      <c r="C48" s="19" t="n"/>
-      <c r="D48" s="19" t="n"/>
-      <c r="E48" s="19" t="n"/>
+      <c r="B48" s="19" t="n">
+        <v>47822.2</v>
+      </c>
+      <c r="C48" s="19" t="n">
+        <v>72199.42999999999</v>
+      </c>
+      <c r="D48" s="19" t="n">
+        <v>74776.71000000001</v>
+      </c>
+      <c r="E48" s="19" t="n">
+        <v>132537.33</v>
+      </c>
       <c r="F48" s="16">
         <f>SUM(F43:F47)</f>
         <v/>
@@ -2113,10 +2455,18 @@
           <t xml:space="preserve">  Client Payables</t>
         </is>
       </c>
-      <c r="B51" s="12" t="n"/>
-      <c r="C51" s="12" t="n"/>
-      <c r="D51" s="12" t="n"/>
-      <c r="E51" s="12" t="n"/>
+      <c r="B51" s="12" t="n">
+        <v>22763.81</v>
+      </c>
+      <c r="C51" s="12" t="n">
+        <v>40668.1</v>
+      </c>
+      <c r="D51" s="12" t="n">
+        <v>40715.07</v>
+      </c>
+      <c r="E51" s="12" t="n">
+        <v>71969.8</v>
+      </c>
       <c r="F51" s="13" t="n"/>
       <c r="G51" s="13" t="n"/>
       <c r="H51" s="13" t="n"/>
@@ -2129,10 +2479,18 @@
           <t xml:space="preserve">  Borrowings (MTF funded)</t>
         </is>
       </c>
-      <c r="B52" s="12" t="n"/>
-      <c r="C52" s="12" t="n"/>
-      <c r="D52" s="12" t="n"/>
-      <c r="E52" s="12" t="n"/>
+      <c r="B52" s="12" t="n">
+        <v>11713.79</v>
+      </c>
+      <c r="C52" s="12" t="n">
+        <v>12577.32</v>
+      </c>
+      <c r="D52" s="12" t="n">
+        <v>7871.86</v>
+      </c>
+      <c r="E52" s="12" t="n">
+        <v>25411.22</v>
+      </c>
       <c r="F52" s="13" t="n"/>
       <c r="G52" s="13" t="n"/>
       <c r="H52" s="13" t="n"/>
@@ -2145,10 +2503,18 @@
           <t xml:space="preserve">  Other Current Liabilities</t>
         </is>
       </c>
-      <c r="B53" s="12" t="n"/>
-      <c r="C53" s="12" t="n"/>
-      <c r="D53" s="12" t="n"/>
-      <c r="E53" s="12" t="n"/>
+      <c r="B53" s="12" t="n">
+        <v>2323.83</v>
+      </c>
+      <c r="C53" s="12" t="n">
+        <v>3110.24</v>
+      </c>
+      <c r="D53" s="12" t="n">
+        <v>4574.2</v>
+      </c>
+      <c r="E53" s="12" t="n">
+        <v>4771.28</v>
+      </c>
       <c r="F53" s="13" t="n"/>
       <c r="G53" s="13" t="n"/>
       <c r="H53" s="13" t="n"/>
@@ -2161,10 +2527,18 @@
           <t>Total Liabilities</t>
         </is>
       </c>
-      <c r="B54" s="19" t="n"/>
-      <c r="C54" s="19" t="n"/>
-      <c r="D54" s="19" t="n"/>
-      <c r="E54" s="19" t="n"/>
+      <c r="B54" s="19" t="n">
+        <v>36801.43</v>
+      </c>
+      <c r="C54" s="19" t="n">
+        <v>56355.66</v>
+      </c>
+      <c r="D54" s="19" t="n">
+        <v>53161.13</v>
+      </c>
+      <c r="E54" s="19" t="n">
+        <v>102152.3</v>
+      </c>
       <c r="F54" s="16">
         <f>SUM(F51:F53)</f>
         <v/>
@@ -2193,10 +2567,18 @@
           <t xml:space="preserve">  Share Capital</t>
         </is>
       </c>
-      <c r="B56" s="12" t="n"/>
-      <c r="C56" s="12" t="n"/>
-      <c r="D56" s="12" t="n"/>
-      <c r="E56" s="12" t="n"/>
+      <c r="B56" s="12" t="n">
+        <v>818.27</v>
+      </c>
+      <c r="C56" s="12" t="n">
+        <v>828.59</v>
+      </c>
+      <c r="D56" s="12" t="n">
+        <v>834.2</v>
+      </c>
+      <c r="E56" s="12" t="n">
+        <v>840.08</v>
+      </c>
       <c r="F56" s="13" t="n"/>
       <c r="G56" s="13" t="n"/>
       <c r="H56" s="13" t="n"/>
@@ -2209,10 +2591,18 @@
           <t xml:space="preserve">  Reserves &amp; Surplus</t>
         </is>
       </c>
-      <c r="B57" s="12" t="n"/>
-      <c r="C57" s="12" t="n"/>
-      <c r="D57" s="12" t="n"/>
-      <c r="E57" s="12" t="n"/>
+      <c r="B57" s="12" t="n">
+        <v>10202.5</v>
+      </c>
+      <c r="C57" s="12" t="n">
+        <v>15015.18</v>
+      </c>
+      <c r="D57" s="12" t="n">
+        <v>20781.38</v>
+      </c>
+      <c r="E57" s="12" t="n">
+        <v>29545.95</v>
+      </c>
       <c r="F57" s="13">
         <f>E57+F36</f>
         <v/>
@@ -2240,10 +2630,18 @@
           <t>Total Equity</t>
         </is>
       </c>
-      <c r="B58" s="19" t="n"/>
-      <c r="C58" s="19" t="n"/>
-      <c r="D58" s="19" t="n"/>
-      <c r="E58" s="19" t="n"/>
+      <c r="B58" s="19" t="n">
+        <v>11020.77</v>
+      </c>
+      <c r="C58" s="19" t="n">
+        <v>15843.77</v>
+      </c>
+      <c r="D58" s="19" t="n">
+        <v>21615.58</v>
+      </c>
+      <c r="E58" s="19" t="n">
+        <v>30385.03</v>
+      </c>
       <c r="F58" s="16">
         <f>F56+F57</f>
         <v/>
@@ -2271,10 +2669,18 @@
           <t>Total Liabilities + Equity</t>
         </is>
       </c>
-      <c r="B59" s="19" t="n"/>
-      <c r="C59" s="19" t="n"/>
-      <c r="D59" s="19" t="n"/>
-      <c r="E59" s="19" t="n"/>
+      <c r="B59" s="19" t="n">
+        <v>47822.2</v>
+      </c>
+      <c r="C59" s="19" t="n">
+        <v>72199.42999999999</v>
+      </c>
+      <c r="D59" s="19" t="n">
+        <v>74776.71000000001</v>
+      </c>
+      <c r="E59" s="19" t="n">
+        <v>132537.33</v>
+      </c>
       <c r="F59" s="16">
         <f>F54+F58</f>
         <v/>
@@ -2302,6 +2708,16 @@
           <t>CASH FLOW STATEMENT</t>
         </is>
       </c>
+      <c r="B62" s="72" t="n"/>
+      <c r="C62" s="72" t="n"/>
+      <c r="D62" s="72" t="n"/>
+      <c r="E62" s="72" t="n"/>
+      <c r="F62" s="72" t="n"/>
+      <c r="G62" s="72" t="n"/>
+      <c r="H62" s="72" t="n"/>
+      <c r="I62" s="72" t="n"/>
+      <c r="J62" s="72" t="n"/>
+      <c r="K62" s="73" t="n"/>
     </row>
     <row r="63" ht="16" customHeight="1">
       <c r="A63" s="11" t="inlineStr">
@@ -2434,10 +2850,18 @@
           <t xml:space="preserve">  CapEx</t>
         </is>
       </c>
-      <c r="B68" s="12" t="n"/>
-      <c r="C68" s="12" t="n"/>
-      <c r="D68" s="12" t="n"/>
-      <c r="E68" s="12" t="n"/>
+      <c r="B68" s="12" t="n">
+        <v>-142.86</v>
+      </c>
+      <c r="C68" s="12" t="n">
+        <v>-697.48</v>
+      </c>
+      <c r="D68" s="12" t="n">
+        <v>-1141.61</v>
+      </c>
+      <c r="E68" s="12" t="n">
+        <v>-2075.05</v>
+      </c>
       <c r="F68" s="13">
         <f>-F23*F15</f>
         <v/>
@@ -2497,10 +2921,18 @@
           <t xml:space="preserve">  Dividends Paid</t>
         </is>
       </c>
-      <c r="B71" s="12" t="n"/>
-      <c r="C71" s="12" t="n"/>
-      <c r="D71" s="12" t="n"/>
-      <c r="E71" s="12" t="n"/>
+      <c r="B71" s="12" t="n">
+        <v>-426.58</v>
+      </c>
+      <c r="C71" s="12" t="n">
+        <v>-1562</v>
+      </c>
+      <c r="D71" s="12" t="n">
+        <v>-2225</v>
+      </c>
+      <c r="E71" s="12" t="n">
+        <v>-3242.2</v>
+      </c>
       <c r="F71" s="13" t="n"/>
       <c r="G71" s="13" t="n"/>
       <c r="H71" s="13" t="n"/>
@@ -2592,7 +3024,9 @@
           <t xml:space="preserve">  Opening Cash</t>
         </is>
       </c>
-      <c r="B76" s="12" t="n"/>
+      <c r="B76" s="12" t="n">
+        <v>5899.92</v>
+      </c>
       <c r="C76" s="12" t="n"/>
       <c r="D76" s="12" t="n"/>
       <c r="E76" s="12" t="n"/>
@@ -2623,10 +3057,18 @@
           <t>Closing Cash</t>
         </is>
       </c>
-      <c r="B77" s="19" t="n"/>
-      <c r="C77" s="19" t="n"/>
-      <c r="D77" s="19" t="n"/>
-      <c r="E77" s="19" t="n"/>
+      <c r="B77" s="19" t="n">
+        <v>18510.51</v>
+      </c>
+      <c r="C77" s="19" t="n">
+        <v>48749.57</v>
+      </c>
+      <c r="D77" s="19" t="n">
+        <v>54910.83</v>
+      </c>
+      <c r="E77" s="19" t="n">
+        <v>98442.94</v>
+      </c>
       <c r="F77" s="16">
         <f>F76+F75</f>
         <v/>
@@ -2654,6 +3096,16 @@
           <t>SANITY CHECK — CLOSING CASH MUST MATCH BALANCE SHEET CASH</t>
         </is>
       </c>
+      <c r="B79" s="72" t="n"/>
+      <c r="C79" s="72" t="n"/>
+      <c r="D79" s="72" t="n"/>
+      <c r="E79" s="72" t="n"/>
+      <c r="F79" s="72" t="n"/>
+      <c r="G79" s="72" t="n"/>
+      <c r="H79" s="72" t="n"/>
+      <c r="I79" s="72" t="n"/>
+      <c r="J79" s="72" t="n"/>
+      <c r="K79" s="73" t="n"/>
     </row>
     <row r="80" ht="20" customHeight="1">
       <c r="A80" s="14" t="inlineStr">
@@ -2689,31 +3141,31 @@
         </is>
       </c>
       <c r="B82" s="12" t="n">
-        <v>85.5</v>
+        <v>908.5</v>
       </c>
       <c r="C82" s="12" t="n">
-        <v>85.5</v>
+        <v>839.3</v>
       </c>
       <c r="D82" s="12" t="n">
-        <v>85.5</v>
+        <v>847</v>
       </c>
       <c r="E82" s="12" t="n">
-        <v>85.5</v>
+        <v>854.1</v>
       </c>
       <c r="F82" s="12" t="n">
-        <v>85.5</v>
+        <v>908.5</v>
       </c>
       <c r="G82" s="12" t="n">
-        <v>85.5</v>
+        <v>908.5</v>
       </c>
       <c r="H82" s="12" t="n">
-        <v>85.5</v>
+        <v>908.5</v>
       </c>
       <c r="I82" s="12" t="n">
-        <v>85.5</v>
+        <v>908.5</v>
       </c>
       <c r="J82" s="12" t="n">
-        <v>85.5</v>
+        <v>908.5</v>
       </c>
     </row>
   </sheetData>
@@ -2762,6 +3214,11 @@
           <t>DCF VALUATION — Angel One Ltd</t>
         </is>
       </c>
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="73" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -2776,6 +3233,8 @@
           <t>WACC INPUTS</t>
         </is>
       </c>
+      <c r="B4" s="72" t="n"/>
+      <c r="C4" s="73" t="n"/>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="11" t="inlineStr">
@@ -2887,6 +3346,11 @@
           <t>FREE CASH FLOW PROJECTION (LINKED FROM 3-STATEMENT MODEL)</t>
         </is>
       </c>
+      <c r="B16" s="72" t="n"/>
+      <c r="C16" s="72" t="n"/>
+      <c r="D16" s="72" t="n"/>
+      <c r="E16" s="72" t="n"/>
+      <c r="F16" s="73" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -3115,6 +3579,8 @@
           <t>TERMINAL VALUE &amp; ENTERPRISE VALUE</t>
         </is>
       </c>
+      <c r="B26" s="72" t="n"/>
+      <c r="C26" s="73" t="n"/>
     </row>
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
@@ -3187,6 +3653,8 @@
           <t>EQUITY BRIDGE &amp; PRICE TARGET</t>
         </is>
       </c>
+      <c r="B38" s="72" t="n"/>
+      <c r="C38" s="73" t="n"/>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="14" t="inlineStr">
@@ -3205,7 +3673,9 @@
           <t xml:space="preserve">  Less: Net Debt</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr"/>
+      <c r="B40" s="12" t="n">
+        <v>15411</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="14" t="inlineStr">
@@ -3247,7 +3717,7 @@
         </is>
       </c>
       <c r="B44" s="27" t="n">
-        <v>212.12</v>
+        <v>232.6</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
@@ -3315,6 +3785,17 @@
           <t>COMPARABLE COMPANY ANALYSIS — Indian Broking Sector</t>
         </is>
       </c>
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="72" t="n"/>
+      <c r="G1" s="72" t="n"/>
+      <c r="H1" s="72" t="n"/>
+      <c r="I1" s="72" t="n"/>
+      <c r="J1" s="72" t="n"/>
+      <c r="K1" s="72" t="n"/>
+      <c r="L1" s="73" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -3406,13 +3887,27 @@
           <t>ANGELONE</t>
         </is>
       </c>
-      <c r="C4" s="34" t="n"/>
-      <c r="D4" s="34" t="n"/>
-      <c r="E4" s="34" t="n"/>
-      <c r="F4" s="34" t="n"/>
-      <c r="G4" s="34" t="n"/>
-      <c r="H4" s="35" t="n"/>
-      <c r="I4" s="34" t="n"/>
+      <c r="C4" s="34" t="n">
+        <v>210120</v>
+      </c>
+      <c r="D4" s="34" t="n">
+        <v>15411</v>
+      </c>
+      <c r="E4" s="34" t="n">
+        <v>225531</v>
+      </c>
+      <c r="F4" s="34" t="n">
+        <v>42798</v>
+      </c>
+      <c r="G4" s="34" t="n">
+        <v>16990</v>
+      </c>
+      <c r="H4" s="35" t="n">
+        <v>0.397</v>
+      </c>
+      <c r="I4" s="34" t="n">
+        <v>11255</v>
+      </c>
       <c r="J4" s="36">
         <f>E4/G4</f>
         <v/>
@@ -3569,6 +4064,7 @@
           <t>Peer Median (ex-Angel One)</t>
         </is>
       </c>
+      <c r="B11" s="73" t="n"/>
       <c r="C11" s="44">
         <f>MEDIAN(C5:C9)</f>
         <v/>
@@ -3616,6 +4112,10 @@
           <t>IMPLIED VALUATION — ANGEL ONE AT PEER MEDIAN MULTIPLES</t>
         </is>
       </c>
+      <c r="B13" s="72" t="n"/>
+      <c r="C13" s="72" t="n"/>
+      <c r="D13" s="72" t="n"/>
+      <c r="E13" s="73" t="n"/>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="11" t="inlineStr">
@@ -3718,6 +4218,10 @@
           <t>SCENARIO ANALYSIS — Bull / Base / Bear</t>
         </is>
       </c>
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="73" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -3864,6 +4368,9 @@
           <t>SCENARIO OUTPUTS — PRICE TARGETS</t>
         </is>
       </c>
+      <c r="B11" s="72" t="n"/>
+      <c r="C11" s="72" t="n"/>
+      <c r="D11" s="73" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
@@ -3990,6 +4497,17 @@
           <t>SENSITIVITY ANALYSIS — Price Target vs. Key Assumptions</t>
         </is>
       </c>
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="72" t="n"/>
+      <c r="G1" s="72" t="n"/>
+      <c r="H1" s="72" t="n"/>
+      <c r="I1" s="72" t="n"/>
+      <c r="J1" s="72" t="n"/>
+      <c r="K1" s="72" t="n"/>
+      <c r="L1" s="73" t="n"/>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="55" t="inlineStr">
@@ -4004,6 +4522,14 @@
           <t>TABLE 1 — IMPLIED PRICE (₹) VS. WACC × TERMINAL GROWTH RATE</t>
         </is>
       </c>
+      <c r="B4" s="72" t="n"/>
+      <c r="C4" s="72" t="n"/>
+      <c r="D4" s="72" t="n"/>
+      <c r="E4" s="72" t="n"/>
+      <c r="F4" s="72" t="n"/>
+      <c r="G4" s="72" t="n"/>
+      <c r="H4" s="72" t="n"/>
+      <c r="I4" s="73" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="56" t="inlineStr">
@@ -4228,6 +4754,14 @@
           <t>TABLE 2 — IMPLIED UPSIDE (%) VS. REVENUE CAGR × EBITDA MARGIN (FY29E)</t>
         </is>
       </c>
+      <c r="B15" s="72" t="n"/>
+      <c r="C15" s="72" t="n"/>
+      <c r="D15" s="72" t="n"/>
+      <c r="E15" s="72" t="n"/>
+      <c r="F15" s="72" t="n"/>
+      <c r="G15" s="72" t="n"/>
+      <c r="H15" s="72" t="n"/>
+      <c r="I15" s="73" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="56" t="inlineStr">
@@ -4437,6 +4971,13 @@
           <t>ANGEL ONE LTD (NSE: ANGELONE) — EQUITY RESEARCH SUMMARY</t>
         </is>
       </c>
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="72" t="n"/>
+      <c r="G1" s="72" t="n"/>
+      <c r="H1" s="73" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -4451,11 +4992,17 @@
           <t>PRICE TARGET &amp; RATING</t>
         </is>
       </c>
+      <c r="B4" s="72" t="n"/>
+      <c r="C4" s="73" t="n"/>
       <c r="D4" s="6" t="inlineStr">
         <is>
           <t>KEY FINANCIAL METRICS</t>
         </is>
       </c>
+      <c r="E4" s="72" t="n"/>
+      <c r="F4" s="72" t="n"/>
+      <c r="G4" s="72" t="n"/>
+      <c r="H4" s="73" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
@@ -4618,6 +5165,13 @@
           <t>INVESTMENT THESIS</t>
         </is>
       </c>
+      <c r="B14" s="72" t="n"/>
+      <c r="C14" s="72" t="n"/>
+      <c r="D14" s="72" t="n"/>
+      <c r="E14" s="72" t="n"/>
+      <c r="F14" s="72" t="n"/>
+      <c r="G14" s="72" t="n"/>
+      <c r="H14" s="73" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="69" t="inlineStr">
@@ -4627,17 +5181,49 @@
 Current price: ₹212 vs. 52-week high of ₹328. At 19x P/E, the market is pricing in significant structural pressure. The DCF price target determines whether this is a dislocation or fair value.</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="20" customHeight="1"/>
-    <row r="17" ht="20" customHeight="1"/>
-    <row r="18" ht="20" customHeight="1"/>
-    <row r="19" ht="20" customHeight="1"/>
+      <c r="B15" s="74" t="n"/>
+      <c r="C15" s="74" t="n"/>
+      <c r="D15" s="74" t="n"/>
+      <c r="E15" s="74" t="n"/>
+      <c r="F15" s="74" t="n"/>
+      <c r="G15" s="74" t="n"/>
+      <c r="H15" s="75" t="n"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="76" t="n"/>
+      <c r="H16" s="77" t="n"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="76" t="n"/>
+      <c r="H17" s="77" t="n"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="76" t="n"/>
+      <c r="H18" s="77" t="n"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="78" t="n"/>
+      <c r="B19" s="79" t="n"/>
+      <c r="C19" s="79" t="n"/>
+      <c r="D19" s="79" t="n"/>
+      <c r="E19" s="79" t="n"/>
+      <c r="F19" s="79" t="n"/>
+      <c r="G19" s="79" t="n"/>
+      <c r="H19" s="80" t="n"/>
+    </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
           <t>DATA SOURCES</t>
         </is>
       </c>
+      <c r="B21" s="72" t="n"/>
+      <c r="C21" s="72" t="n"/>
+      <c r="D21" s="72" t="n"/>
+      <c r="E21" s="72" t="n"/>
+      <c r="F21" s="72" t="n"/>
+      <c r="G21" s="72" t="n"/>
+      <c r="H21" s="73" t="n"/>
     </row>
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="70" t="inlineStr">
@@ -4645,6 +5231,13 @@
           <t>Angel One Investor Relations: https://www.angelone.in/investor-relations</t>
         </is>
       </c>
+      <c r="B22" s="72" t="n"/>
+      <c r="C22" s="72" t="n"/>
+      <c r="D22" s="72" t="n"/>
+      <c r="E22" s="72" t="n"/>
+      <c r="F22" s="72" t="n"/>
+      <c r="G22" s="72" t="n"/>
+      <c r="H22" s="73" t="n"/>
     </row>
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="70" t="inlineStr">
@@ -4652,6 +5245,13 @@
           <t>BSE Filings (code 543235): https://www.bseindia.com</t>
         </is>
       </c>
+      <c r="B23" s="72" t="n"/>
+      <c r="C23" s="72" t="n"/>
+      <c r="D23" s="72" t="n"/>
+      <c r="E23" s="72" t="n"/>
+      <c r="F23" s="72" t="n"/>
+      <c r="G23" s="72" t="n"/>
+      <c r="H23" s="73" t="n"/>
     </row>
     <row r="24" ht="16" customHeight="1">
       <c r="A24" s="70" t="inlineStr">
@@ -4659,6 +5259,13 @@
           <t>Screener.in: https://www.screener.in/company/ANGELONE/consolidated/</t>
         </is>
       </c>
+      <c r="B24" s="72" t="n"/>
+      <c r="C24" s="72" t="n"/>
+      <c r="D24" s="72" t="n"/>
+      <c r="E24" s="72" t="n"/>
+      <c r="F24" s="72" t="n"/>
+      <c r="G24" s="72" t="n"/>
+      <c r="H24" s="73" t="n"/>
     </row>
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="70" t="inlineStr">
@@ -4666,6 +5273,13 @@
           <t>SEBI monthly broker data: https://www.sebi.gov.in</t>
         </is>
       </c>
+      <c r="B25" s="72" t="n"/>
+      <c r="C25" s="72" t="n"/>
+      <c r="D25" s="72" t="n"/>
+      <c r="E25" s="72" t="n"/>
+      <c r="F25" s="72" t="n"/>
+      <c r="G25" s="72" t="n"/>
+      <c r="H25" s="73" t="n"/>
     </row>
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="70" t="inlineStr">
@@ -4673,6 +5287,13 @@
           <t>NSE monthly market data: https://www.nseindia.com</t>
         </is>
       </c>
+      <c r="B26" s="72" t="n"/>
+      <c r="C26" s="72" t="n"/>
+      <c r="D26" s="72" t="n"/>
+      <c r="E26" s="72" t="n"/>
+      <c r="F26" s="72" t="n"/>
+      <c r="G26" s="72" t="n"/>
+      <c r="H26" s="73" t="n"/>
     </row>
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="70" t="inlineStr">
@@ -4680,6 +5301,13 @@
           <t>AMFI data: https://www.amfiindia.com</t>
         </is>
       </c>
+      <c r="B27" s="72" t="n"/>
+      <c r="C27" s="72" t="n"/>
+      <c r="D27" s="72" t="n"/>
+      <c r="E27" s="72" t="n"/>
+      <c r="F27" s="72" t="n"/>
+      <c r="G27" s="72" t="n"/>
+      <c r="H27" s="73" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
@@ -4687,6 +5315,13 @@
           <t>KEY RISKS</t>
         </is>
       </c>
+      <c r="B29" s="72" t="n"/>
+      <c r="C29" s="72" t="n"/>
+      <c r="D29" s="72" t="n"/>
+      <c r="E29" s="72" t="n"/>
+      <c r="F29" s="72" t="n"/>
+      <c r="G29" s="72" t="n"/>
+      <c r="H29" s="73" t="n"/>
     </row>
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="71" t="inlineStr">
@@ -4694,6 +5329,13 @@
           <t>• Regulatory: Further SEBI F&amp;O tightening could structurally reduce retail participation and brokerage take rates</t>
         </is>
       </c>
+      <c r="B30" s="72" t="n"/>
+      <c r="C30" s="72" t="n"/>
+      <c r="D30" s="72" t="n"/>
+      <c r="E30" s="72" t="n"/>
+      <c r="F30" s="72" t="n"/>
+      <c r="G30" s="72" t="n"/>
+      <c r="H30" s="73" t="n"/>
     </row>
     <row r="31" ht="22" customHeight="1">
       <c r="A31" s="71" t="inlineStr">
@@ -4701,6 +5343,13 @@
           <t>• Competition: Zerodha, Groww maintain strong brand loyalty; market share defence required</t>
         </is>
       </c>
+      <c r="B31" s="72" t="n"/>
+      <c r="C31" s="72" t="n"/>
+      <c r="D31" s="72" t="n"/>
+      <c r="E31" s="72" t="n"/>
+      <c r="F31" s="72" t="n"/>
+      <c r="G31" s="72" t="n"/>
+      <c r="H31" s="73" t="n"/>
     </row>
     <row r="32" ht="22" customHeight="1">
       <c r="A32" s="71" t="inlineStr">
@@ -4708,6 +5357,13 @@
           <t>• Margin compression: EBITDA fell from 46.8% (FY24) to 32.5% (Q4 FY25) — recovery trajectory uncertain</t>
         </is>
       </c>
+      <c r="B32" s="72" t="n"/>
+      <c r="C32" s="72" t="n"/>
+      <c r="D32" s="72" t="n"/>
+      <c r="E32" s="72" t="n"/>
+      <c r="F32" s="72" t="n"/>
+      <c r="G32" s="72" t="n"/>
+      <c r="H32" s="73" t="n"/>
     </row>
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="71" t="inlineStr">
@@ -4715,6 +5371,13 @@
           <t>• Market dependency: Revenue heavily correlated to market volumes (downturns = significant PAT decline)</t>
         </is>
       </c>
+      <c r="B33" s="72" t="n"/>
+      <c r="C33" s="72" t="n"/>
+      <c r="D33" s="72" t="n"/>
+      <c r="E33" s="72" t="n"/>
+      <c r="F33" s="72" t="n"/>
+      <c r="G33" s="72" t="n"/>
+      <c r="H33" s="73" t="n"/>
     </row>
     <row r="34" ht="22" customHeight="1">
       <c r="A34" s="71" t="inlineStr">
@@ -4722,6 +5385,13 @@
           <t>• MTF book risk: Margin lending creates credit exposure in volatile markets</t>
         </is>
       </c>
+      <c r="B34" s="72" t="n"/>
+      <c r="C34" s="72" t="n"/>
+      <c r="D34" s="72" t="n"/>
+      <c r="E34" s="72" t="n"/>
+      <c r="F34" s="72" t="n"/>
+      <c r="G34" s="72" t="n"/>
+      <c r="H34" s="73" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="19">

</xml_diff>